<commit_message>
Added IRetryAnalyzer to rerun failed test cases and added condition in the Login test to handle retryAnalyzer
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sathi\SDET JAVA\Java automation\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7FC1E62-E3FD-478B-BEA5-5017CE716874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E8D225-9E1B-49CA-B9F7-3BFA0155048E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>userName</t>
   </si>
@@ -33,6 +33,9 @@
     <t>password</t>
   </si>
   <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
     <t>standard_user</t>
   </si>
   <si>
@@ -42,7 +45,16 @@
     <t>performance_glitch_user</t>
   </si>
   <si>
-    <t>secret_sauce</t>
+    <t>expectedResult</t>
+  </si>
+  <si>
+    <t>standard_user1</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
 </sst>
 </file>
@@ -360,43 +372,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
     <col min="2" max="2" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed the hard code number max no attempts and current attempts value in the Retry Analyzer class from com.ui.listeners package
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sathi\SDET JAVA\Java automation\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E8D225-9E1B-49CA-B9F7-3BFA0155048E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1825671-A4CF-4D97-BD81-5298062DA9B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,13 +48,13 @@
     <t>expectedResult</t>
   </si>
   <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
     <t>standard_user1</t>
-  </si>
-  <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>FAIL</t>
   </si>
 </sst>
 </file>
@@ -399,7 +399,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -410,7 +410,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -421,18 +421,18 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>